<commit_message>
Daily job match 2026-08-04
</commit_message>
<xml_diff>
--- a/output/matches_2026-08-04.xlsx
+++ b/output/matches_2026-08-04.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.adzuna.com/land/ad/5748993355?se=cGThIBSQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=5B16C3053C01862EF92DC23FA2C9085FF09628CB</t>
+          <t>https://www.adzuna.com/land/ad/5748993355?se=rJe_lxiQ8RG5JrYntIBpaQ&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=5B16C3053C01862EF92DC23FA2C9085FF09628CB</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.adzuna.com/land/ad/5675791814?se=TCZgIhSQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=610E7E521ED8D4538CFE5FB51E84C0B508A35CF8</t>
+          <t>https://www.adzuna.com/land/ad/5675791814?se=HioUmRiQ8RGJSr6zDeCjPA&amp;utm_medium=api&amp;utm_source=c998f847&amp;v=610E7E521ED8D4538CFE5FB51E84C0B508A35CF8</t>
         </is>
       </c>
     </row>

</xml_diff>